<commit_message>
kết nối test thành công Login
</commit_message>
<xml_diff>
--- a/test/appium_tests/result/result_login.xlsx
+++ b/test/appium_tests/result/result_login.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,22 +451,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Failed Login</t>
+          <t>Test 7</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>wrong@example.com</t>
+          <t>khai@gmail.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>wrongpassword</t>
+          <t>123456</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Đăng nhập không thành công: Exception: Đăng nhập không thành công</t>
+          <t>Đăng nhập thành công (không có thông báo lỗi)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -476,129 +476,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2025-04-20 15:26:42</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Successful Login</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>khai@gmail.com</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Đăng nhập thành công (không có thông báo lỗi)</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2025-04-20 15:27:49</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Failed Login</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>wrong@example.com</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>wrongpassword</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Đăng nhập không thành công: Exception: Đăng nhập không thành công</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2025-04-21 19:57:25</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Successful Login</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>khai@gmail.com</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Đăng nhập thành công (không có thông báo lỗi)</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2025-04-21 19:58:13</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Test 1</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="n">
-        <v>123456</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Lỗi: object of type 'int' has no len()</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>2025-04-22 01:42:40</t>
+          <t>2025-04-22 02:42:05</t>
         </is>
       </c>
     </row>

</xml_diff>